<commit_message>
feat: add safe full database reset and seeding
</commit_message>
<xml_diff>
--- a/reference_data.xlsx
+++ b/reference_data.xlsx
@@ -1,36 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LYS\Desktop\ASF\project_2\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C3DD989-6BCE-453F-B2B2-B4619C217716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24120" yWindow="-120" windowWidth="24240" windowHeight="13140" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-24120" yWindow="-120" windowWidth="24240" windowHeight="13140" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="positions" sheetId="1" r:id="rId1"/>
-    <sheet name="persons" sheetId="2" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="positions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="persons" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="seed_config" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -352,31 +333,32 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Times New Roman"/>
+      <charset val="204"/>
+      <family val="1"/>
+      <color theme="1"/>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
     </font>
     <font>
-      <sz val="11"/>
       <name val="Consolas"/>
       <family val="3"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -415,32 +397,92 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Звичайний" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -1216,441 +1258,1280 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF7B9615-41E1-4B21-8921-1A96F23A385D}">
-  <dimension ref="A1:I16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="4" width="16.5703125" customWidth="1"/>
-    <col min="5" max="5" width="18.5703125" style="3" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" customWidth="1"/>
-    <col min="8" max="8" width="12.7109375" customWidth="1"/>
-    <col min="9" max="9" width="21.140625" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AS6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>103</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="I1" t="s">
-        <v>97</v>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>surname</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>patronymic</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>tax_number</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>birth_day</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>birth_month</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>birth_year</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>sex</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>birth_country</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>birth_region</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
+          <t>birth_district</t>
+        </is>
+      </c>
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>birth_community</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>birth_settlement</t>
+        </is>
+      </c>
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>birth_settlement_type</t>
+        </is>
+      </c>
+      <c r="P1" s="5" t="inlineStr">
+        <is>
+          <t>registration_country</t>
+        </is>
+      </c>
+      <c r="Q1" s="5" t="inlineStr">
+        <is>
+          <t>registration_region</t>
+        </is>
+      </c>
+      <c r="R1" s="5" t="inlineStr">
+        <is>
+          <t>registration_district</t>
+        </is>
+      </c>
+      <c r="S1" s="5" t="inlineStr">
+        <is>
+          <t>registration_community</t>
+        </is>
+      </c>
+      <c r="T1" s="5" t="inlineStr">
+        <is>
+          <t>registration_settlement</t>
+        </is>
+      </c>
+      <c r="U1" s="5" t="inlineStr">
+        <is>
+          <t>registration_settlement_type</t>
+        </is>
+      </c>
+      <c r="V1" s="5" t="inlineStr">
+        <is>
+          <t>registration_street</t>
+        </is>
+      </c>
+      <c r="W1" s="5" t="inlineStr">
+        <is>
+          <t>registration_street_type</t>
+        </is>
+      </c>
+      <c r="X1" s="5" t="inlineStr">
+        <is>
+          <t>registration_house</t>
+        </is>
+      </c>
+      <c r="Y1" s="5" t="inlineStr">
+        <is>
+          <t>registration_corps</t>
+        </is>
+      </c>
+      <c r="Z1" s="5" t="inlineStr">
+        <is>
+          <t>registration_building</t>
+        </is>
+      </c>
+      <c r="AA1" s="5" t="inlineStr">
+        <is>
+          <t>registration_apartment</t>
+        </is>
+      </c>
+      <c r="AB1" s="5" t="inlineStr">
+        <is>
+          <t>registration_room</t>
+        </is>
+      </c>
+      <c r="AC1" s="5" t="inlineStr">
+        <is>
+          <t>registration_postal_code</t>
+        </is>
+      </c>
+      <c r="AD1" s="5" t="inlineStr">
+        <is>
+          <t>registration_note</t>
+        </is>
+      </c>
+      <c r="AE1" s="5" t="inlineStr">
+        <is>
+          <t>actual_country</t>
+        </is>
+      </c>
+      <c r="AF1" s="5" t="inlineStr">
+        <is>
+          <t>actual_region</t>
+        </is>
+      </c>
+      <c r="AG1" s="5" t="inlineStr">
+        <is>
+          <t>actual_district</t>
+        </is>
+      </c>
+      <c r="AH1" s="5" t="inlineStr">
+        <is>
+          <t>actual_community</t>
+        </is>
+      </c>
+      <c r="AI1" s="5" t="inlineStr">
+        <is>
+          <t>actual_settlement</t>
+        </is>
+      </c>
+      <c r="AJ1" s="5" t="inlineStr">
+        <is>
+          <t>actual_settlement_type</t>
+        </is>
+      </c>
+      <c r="AK1" s="5" t="inlineStr">
+        <is>
+          <t>actual_street</t>
+        </is>
+      </c>
+      <c r="AL1" s="5" t="inlineStr">
+        <is>
+          <t>actual_street_type</t>
+        </is>
+      </c>
+      <c r="AM1" s="5" t="inlineStr">
+        <is>
+          <t>actual_house</t>
+        </is>
+      </c>
+      <c r="AN1" s="5" t="inlineStr">
+        <is>
+          <t>actual_corps</t>
+        </is>
+      </c>
+      <c r="AO1" s="5" t="inlineStr">
+        <is>
+          <t>actual_building</t>
+        </is>
+      </c>
+      <c r="AP1" s="5" t="inlineStr">
+        <is>
+          <t>actual_apartment</t>
+        </is>
+      </c>
+      <c r="AQ1" s="5" t="inlineStr">
+        <is>
+          <t>actual_room</t>
+        </is>
+      </c>
+      <c r="AR1" s="5" t="inlineStr">
+        <is>
+          <t>actual_postal_code</t>
+        </is>
+      </c>
+      <c r="AS1" s="5" t="inlineStr">
+        <is>
+          <t>actual_note</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E2" s="3">
-        <v>2849310235</v>
-      </c>
-      <c r="F2">
-        <v>14</v>
-      </c>
-      <c r="G2">
-        <v>5</v>
-      </c>
-      <c r="H2">
-        <v>1988</v>
-      </c>
-      <c r="I2" t="s">
-        <v>84</v>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Прізвище</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Ім’я</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>По батькові</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>РНОКПП</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>День народження</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Місяць народження</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Рік народження</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Звання</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>Стать</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Країна</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>Область / регіон</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>Район</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>Територіальна громада</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>Населений пункт</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>Тип населеного пункту</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>Країна</t>
+        </is>
+      </c>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>Область / регіон</t>
+        </is>
+      </c>
+      <c r="R2" s="5" t="inlineStr">
+        <is>
+          <t>Район</t>
+        </is>
+      </c>
+      <c r="S2" s="5" t="inlineStr">
+        <is>
+          <t>Територіальна громада</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="inlineStr">
+        <is>
+          <t>Населений пункт</t>
+        </is>
+      </c>
+      <c r="U2" s="5" t="inlineStr">
+        <is>
+          <t>Тип населеного пункту</t>
+        </is>
+      </c>
+      <c r="V2" s="5" t="inlineStr">
+        <is>
+          <t>Назва вулиці</t>
+        </is>
+      </c>
+      <c r="W2" s="5" t="inlineStr">
+        <is>
+          <t>Тип вулиці</t>
+        </is>
+      </c>
+      <c r="X2" s="5" t="inlineStr">
+        <is>
+          <t>Будинок</t>
+        </is>
+      </c>
+      <c r="Y2" s="5" t="inlineStr">
+        <is>
+          <t>Корпус</t>
+        </is>
+      </c>
+      <c r="Z2" s="5" t="inlineStr">
+        <is>
+          <t>Будівля / споруда</t>
+        </is>
+      </c>
+      <c r="AA2" s="5" t="inlineStr">
+        <is>
+          <t>Квартира</t>
+        </is>
+      </c>
+      <c r="AB2" s="5" t="inlineStr">
+        <is>
+          <t>Кімната</t>
+        </is>
+      </c>
+      <c r="AC2" s="5" t="inlineStr">
+        <is>
+          <t>Поштовий індекс</t>
+        </is>
+      </c>
+      <c r="AD2" s="5" t="inlineStr">
+        <is>
+          <t>Уточнення</t>
+        </is>
+      </c>
+      <c r="AE2" s="5" t="inlineStr">
+        <is>
+          <t>Країна</t>
+        </is>
+      </c>
+      <c r="AF2" s="5" t="inlineStr">
+        <is>
+          <t>Область / регіон</t>
+        </is>
+      </c>
+      <c r="AG2" s="5" t="inlineStr">
+        <is>
+          <t>Район</t>
+        </is>
+      </c>
+      <c r="AH2" s="5" t="inlineStr">
+        <is>
+          <t>Територіальна громада</t>
+        </is>
+      </c>
+      <c r="AI2" s="5" t="inlineStr">
+        <is>
+          <t>Населений пункт</t>
+        </is>
+      </c>
+      <c r="AJ2" s="5" t="inlineStr">
+        <is>
+          <t>Тип населеного пункту</t>
+        </is>
+      </c>
+      <c r="AK2" s="5" t="inlineStr">
+        <is>
+          <t>Назва вулиці</t>
+        </is>
+      </c>
+      <c r="AL2" s="5" t="inlineStr">
+        <is>
+          <t>Тип вулиці</t>
+        </is>
+      </c>
+      <c r="AM2" s="5" t="inlineStr">
+        <is>
+          <t>Будинок</t>
+        </is>
+      </c>
+      <c r="AN2" s="5" t="inlineStr">
+        <is>
+          <t>Корпус</t>
+        </is>
+      </c>
+      <c r="AO2" s="5" t="inlineStr">
+        <is>
+          <t>Будівля / споруда</t>
+        </is>
+      </c>
+      <c r="AP2" s="5" t="inlineStr">
+        <is>
+          <t>Квартира</t>
+        </is>
+      </c>
+      <c r="AQ2" s="5" t="inlineStr">
+        <is>
+          <t>Кімната</t>
+        </is>
+      </c>
+      <c r="AR2" s="5" t="inlineStr">
+        <is>
+          <t>Поштовий індекс</t>
+        </is>
+      </c>
+      <c r="AS2" s="5" t="inlineStr">
+        <is>
+          <t>Уточнення</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D3" t="s">
-        <v>44</v>
-      </c>
-      <c r="E3" s="3">
-        <v>3124508914</v>
-      </c>
-      <c r="G3">
-        <v>11</v>
-      </c>
-      <c r="H3">
-        <v>1995</v>
-      </c>
-      <c r="I3" t="s">
-        <v>85</v>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Тестенко</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Олександр</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Тестович</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>0000000001</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>1990</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>солдат</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>male</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>Дніпропетровська</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Криворізький</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>Криворізька</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>Кривий Ріг</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>місто</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>Дніпропетровська</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>Криворізький</t>
+        </is>
+      </c>
+      <c r="S3" s="5" t="inlineStr">
+        <is>
+          <t>Криворізька</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
+        <is>
+          <t>Кривий Ріг</t>
+        </is>
+      </c>
+      <c r="U3" s="5" t="inlineStr">
+        <is>
+          <t>місто</t>
+        </is>
+      </c>
+      <c r="V3" s="5" t="inlineStr">
+        <is>
+          <t>Бруно</t>
+        </is>
+      </c>
+      <c r="W3" s="5" t="inlineStr">
+        <is>
+          <t>вулиця</t>
+        </is>
+      </c>
+      <c r="X3" s="5" t="inlineStr">
+        <is>
+          <t>01А/2</t>
+        </is>
+      </c>
+      <c r="Y3" s="5" t="n"/>
+      <c r="Z3" s="5" t="n"/>
+      <c r="AA3" s="5" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="AB3" s="5" t="n"/>
+      <c r="AC3" s="5" t="n"/>
+      <c r="AD3" s="5" t="inlineStr">
+        <is>
+          <t>Вигаданий навчальний приклад; не є адресою реальної особи</t>
+        </is>
+      </c>
+      <c r="AE3" s="5" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="AF3" s="5" t="inlineStr">
+        <is>
+          <t>Дніпропетровська</t>
+        </is>
+      </c>
+      <c r="AG3" s="5" t="inlineStr">
+        <is>
+          <t>Криворізький</t>
+        </is>
+      </c>
+      <c r="AH3" s="5" t="inlineStr">
+        <is>
+          <t>Криворізька</t>
+        </is>
+      </c>
+      <c r="AI3" s="5" t="inlineStr">
+        <is>
+          <t>Кривий Ріг</t>
+        </is>
+      </c>
+      <c r="AJ3" s="5" t="inlineStr">
+        <is>
+          <t>місто</t>
+        </is>
+      </c>
+      <c r="AK3" s="5" t="inlineStr">
+        <is>
+          <t>Бруно</t>
+        </is>
+      </c>
+      <c r="AL3" s="5" t="inlineStr">
+        <is>
+          <t>вулиця</t>
+        </is>
+      </c>
+      <c r="AM3" s="5" t="inlineStr">
+        <is>
+          <t>01А/2</t>
+        </is>
+      </c>
+      <c r="AN3" s="5" t="n"/>
+      <c r="AO3" s="5" t="n"/>
+      <c r="AP3" s="5" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="AQ3" s="5" t="n"/>
+      <c r="AR3" s="5" t="n"/>
+      <c r="AS3" s="5" t="inlineStr">
+        <is>
+          <t>Вигаданий навчальний приклад; не є адресою реальної особи</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E4" s="3">
-        <v>2981704562</v>
-      </c>
-      <c r="F4">
-        <v>23</v>
-      </c>
-      <c r="G4">
-        <v>8</v>
-      </c>
-      <c r="I4" t="s">
-        <v>86</v>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Тестенко</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Олена</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Тестівна</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>0000000002</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>1990</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>солдат</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>female</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Дніпропетровська</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Криворізький</t>
+        </is>
+      </c>
+      <c r="M4" s="5" t="inlineStr">
+        <is>
+          <t>Криворізька</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
+        <is>
+          <t>Кривий Ріг</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>місто</t>
+        </is>
+      </c>
+      <c r="P4" s="5" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t>Дніпропетровська</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
+        <is>
+          <t>Криворізький</t>
+        </is>
+      </c>
+      <c r="S4" s="5" t="inlineStr">
+        <is>
+          <t>Криворізька</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr">
+        <is>
+          <t>Кривий Ріг</t>
+        </is>
+      </c>
+      <c r="U4" s="5" t="inlineStr">
+        <is>
+          <t>місто</t>
+        </is>
+      </c>
+      <c r="V4" s="5" t="inlineStr">
+        <is>
+          <t>Бруно</t>
+        </is>
+      </c>
+      <c r="W4" s="5" t="inlineStr">
+        <is>
+          <t>вулиця</t>
+        </is>
+      </c>
+      <c r="X4" s="5" t="inlineStr">
+        <is>
+          <t>01А/2</t>
+        </is>
+      </c>
+      <c r="Y4" s="5" t="n"/>
+      <c r="Z4" s="5" t="n"/>
+      <c r="AA4" s="5" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="AB4" s="5" t="n"/>
+      <c r="AC4" s="5" t="n"/>
+      <c r="AD4" s="5" t="inlineStr">
+        <is>
+          <t>Вигаданий навчальний приклад; не є адресою реальної особи</t>
+        </is>
+      </c>
+      <c r="AE4" s="5" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="AF4" s="5" t="inlineStr">
+        <is>
+          <t>Дніпропетровська</t>
+        </is>
+      </c>
+      <c r="AG4" s="5" t="inlineStr">
+        <is>
+          <t>Криворізький</t>
+        </is>
+      </c>
+      <c r="AH4" s="5" t="inlineStr">
+        <is>
+          <t>Криворізька</t>
+        </is>
+      </c>
+      <c r="AI4" s="5" t="inlineStr">
+        <is>
+          <t>Кривий Ріг</t>
+        </is>
+      </c>
+      <c r="AJ4" s="5" t="inlineStr">
+        <is>
+          <t>місто</t>
+        </is>
+      </c>
+      <c r="AK4" s="5" t="inlineStr">
+        <is>
+          <t>Бруно</t>
+        </is>
+      </c>
+      <c r="AL4" s="5" t="inlineStr">
+        <is>
+          <t>вулиця</t>
+        </is>
+      </c>
+      <c r="AM4" s="5" t="inlineStr">
+        <is>
+          <t>99Б</t>
+        </is>
+      </c>
+      <c r="AN4" s="5" t="n"/>
+      <c r="AO4" s="5" t="n"/>
+      <c r="AP4" s="5" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="AQ4" s="5" t="n"/>
+      <c r="AR4" s="5" t="n"/>
+      <c r="AS4" s="5" t="inlineStr">
+        <is>
+          <t>Вигаданий навчальний приклад; не є адресою реальної особи</t>
+        </is>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C5" t="s">
-        <v>49</v>
-      </c>
-      <c r="D5" t="s">
-        <v>50</v>
-      </c>
-      <c r="E5" s="3">
-        <v>3451209871</v>
-      </c>
-      <c r="F5">
-        <v>9</v>
-      </c>
-      <c r="H5">
-        <v>2001</v>
-      </c>
-      <c r="I5" t="s">
-        <v>87</v>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Тестенко</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Іван</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Тестович</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>0000000003</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>1990</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>солдат</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>male</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr"/>
+      <c r="K5" s="5" t="inlineStr"/>
+      <c r="L5" s="5" t="inlineStr"/>
+      <c r="M5" s="5" t="inlineStr"/>
+      <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>Навчальне Селище Без Довідника</t>
+        </is>
+      </c>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>місто</t>
+        </is>
+      </c>
+      <c r="P5" s="5" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>Дніпропетровська</t>
+        </is>
+      </c>
+      <c r="R5" s="5" t="inlineStr">
+        <is>
+          <t>Криворізький</t>
+        </is>
+      </c>
+      <c r="S5" s="5" t="inlineStr">
+        <is>
+          <t>Криворізька</t>
+        </is>
+      </c>
+      <c r="T5" s="5" t="inlineStr">
+        <is>
+          <t>Кривий Ріг</t>
+        </is>
+      </c>
+      <c r="U5" s="5" t="inlineStr">
+        <is>
+          <t>місто</t>
+        </is>
+      </c>
+      <c r="V5" s="5" t="inlineStr">
+        <is>
+          <t>Бруно</t>
+        </is>
+      </c>
+      <c r="W5" s="5" t="inlineStr">
+        <is>
+          <t>вулиця</t>
+        </is>
+      </c>
+      <c r="X5" s="5" t="inlineStr">
+        <is>
+          <t>01А/2</t>
+        </is>
+      </c>
+      <c r="Y5" s="5" t="n"/>
+      <c r="Z5" s="5" t="n"/>
+      <c r="AA5" s="5" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="AB5" s="5" t="n"/>
+      <c r="AC5" s="5" t="n"/>
+      <c r="AD5" s="5" t="inlineStr">
+        <is>
+          <t>Вигаданий навчальний приклад; не є адресою реальної особи</t>
+        </is>
+      </c>
+      <c r="AE5" s="5" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="AF5" s="5" t="inlineStr">
+        <is>
+          <t>Дніпропетровська</t>
+        </is>
+      </c>
+      <c r="AG5" s="5" t="inlineStr">
+        <is>
+          <t>Криворізький</t>
+        </is>
+      </c>
+      <c r="AH5" s="5" t="inlineStr">
+        <is>
+          <t>Криворізька</t>
+        </is>
+      </c>
+      <c r="AI5" s="5" t="inlineStr">
+        <is>
+          <t>Кривий Ріг</t>
+        </is>
+      </c>
+      <c r="AJ5" s="5" t="inlineStr">
+        <is>
+          <t>місто</t>
+        </is>
+      </c>
+      <c r="AK5" s="5" t="inlineStr">
+        <is>
+          <t>Бруно</t>
+        </is>
+      </c>
+      <c r="AL5" s="5" t="inlineStr">
+        <is>
+          <t>вулиця</t>
+        </is>
+      </c>
+      <c r="AM5" s="5" t="inlineStr">
+        <is>
+          <t>01А/2</t>
+        </is>
+      </c>
+      <c r="AN5" s="5" t="n"/>
+      <c r="AO5" s="5" t="n"/>
+      <c r="AP5" s="5" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="AQ5" s="5" t="n"/>
+      <c r="AR5" s="5" t="n"/>
+      <c r="AS5" s="5" t="inlineStr">
+        <is>
+          <t>Вигаданий навчальний приклад; не є адресою реальної особи</t>
+        </is>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" t="s">
-        <v>52</v>
-      </c>
-      <c r="D6" t="s">
-        <v>53</v>
-      </c>
-      <c r="E6" s="3">
-        <v>2738401923</v>
-      </c>
-      <c r="F6">
-        <v>18</v>
-      </c>
-      <c r="G6">
-        <v>2</v>
-      </c>
-      <c r="H6">
-        <v>1992</v>
-      </c>
-      <c r="I6" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>54</v>
-      </c>
-      <c r="C7" t="s">
-        <v>55</v>
-      </c>
-      <c r="D7" t="s">
-        <v>56</v>
-      </c>
-      <c r="E7" s="3">
-        <v>3210905438</v>
-      </c>
-      <c r="G7">
-        <v>4</v>
-      </c>
-      <c r="I7" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>57</v>
-      </c>
-      <c r="C8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E8" s="3">
-        <v>3048506129</v>
-      </c>
-      <c r="F8">
-        <v>5</v>
-      </c>
-      <c r="G8">
-        <v>12</v>
-      </c>
-      <c r="H8">
-        <v>1985</v>
-      </c>
-      <c r="I8" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>60</v>
-      </c>
-      <c r="C9" t="s">
-        <v>61</v>
-      </c>
-      <c r="D9" t="s">
-        <v>62</v>
-      </c>
-      <c r="E9" s="3">
-        <v>2893407651</v>
-      </c>
-      <c r="H9">
-        <v>1999</v>
-      </c>
-      <c r="I9" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>63</v>
-      </c>
-      <c r="C10" t="s">
-        <v>64</v>
-      </c>
-      <c r="D10" t="s">
-        <v>65</v>
-      </c>
-      <c r="E10" s="3">
-        <v>3362104897</v>
-      </c>
-      <c r="F10">
-        <v>27</v>
-      </c>
-      <c r="I10" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>66</v>
-      </c>
-      <c r="C11" t="s">
-        <v>67</v>
-      </c>
-      <c r="D11" t="s">
-        <v>68</v>
-      </c>
-      <c r="E11" s="3">
-        <v>2674503186</v>
-      </c>
-      <c r="F11">
-        <v>31</v>
-      </c>
-      <c r="G11">
-        <v>7</v>
-      </c>
-      <c r="H11">
-        <v>2003</v>
-      </c>
-      <c r="I11" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>69</v>
-      </c>
-      <c r="C12" t="s">
-        <v>70</v>
-      </c>
-      <c r="D12" t="s">
-        <v>71</v>
-      </c>
-      <c r="E12" s="3">
-        <v>3189205740</v>
-      </c>
-      <c r="F12">
-        <v>12</v>
-      </c>
-      <c r="H12">
-        <v>1990</v>
-      </c>
-      <c r="I12" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s">
-        <v>72</v>
-      </c>
-      <c r="C13" t="s">
-        <v>73</v>
-      </c>
-      <c r="D13" t="s">
-        <v>74</v>
-      </c>
-      <c r="E13" s="3">
-        <v>2940308165</v>
-      </c>
-      <c r="G13">
-        <v>9</v>
-      </c>
-      <c r="H13">
-        <v>2004</v>
-      </c>
-      <c r="I13" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
-        <v>75</v>
-      </c>
-      <c r="C14" t="s">
-        <v>76</v>
-      </c>
-      <c r="D14" t="s">
-        <v>77</v>
-      </c>
-      <c r="E14" s="3">
-        <v>3257109432</v>
-      </c>
-      <c r="F14">
-        <v>25</v>
-      </c>
-      <c r="G14">
-        <v>3</v>
-      </c>
-      <c r="H14">
-        <v>1982</v>
-      </c>
-      <c r="I14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="s">
-        <v>78</v>
-      </c>
-      <c r="C15" t="s">
-        <v>79</v>
-      </c>
-      <c r="D15" t="s">
-        <v>80</v>
-      </c>
-      <c r="E15" s="3">
-        <v>2798406218</v>
-      </c>
-      <c r="F15">
-        <v>8</v>
-      </c>
-      <c r="G15">
-        <v>10</v>
-      </c>
-      <c r="I15" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="s">
-        <v>81</v>
-      </c>
-      <c r="C16" t="s">
-        <v>82</v>
-      </c>
-      <c r="D16" t="s">
-        <v>83</v>
-      </c>
-      <c r="E16" s="3">
-        <v>3012504983</v>
-      </c>
-      <c r="H16">
-        <v>1997</v>
-      </c>
-      <c r="I16" t="s">
-        <v>94</v>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Тестенко</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Анна</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Тестівна</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>0000000004</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>1990</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>солдат</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>female</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="inlineStr"/>
+      <c r="M6" s="5" t="inlineStr"/>
+      <c r="N6" s="5" t="inlineStr"/>
+      <c r="O6" s="5" t="inlineStr"/>
+      <c r="P6" s="5" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="Q6" s="5" t="inlineStr">
+        <is>
+          <t>Дніпропетровська</t>
+        </is>
+      </c>
+      <c r="R6" s="5" t="inlineStr">
+        <is>
+          <t>Криворізький</t>
+        </is>
+      </c>
+      <c r="S6" s="5" t="inlineStr">
+        <is>
+          <t>Криворізька</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr">
+        <is>
+          <t>Кривий Ріг</t>
+        </is>
+      </c>
+      <c r="U6" s="5" t="inlineStr">
+        <is>
+          <t>місто</t>
+        </is>
+      </c>
+      <c r="V6" s="5" t="inlineStr">
+        <is>
+          <t>Бруно</t>
+        </is>
+      </c>
+      <c r="W6" s="5" t="inlineStr">
+        <is>
+          <t>вулиця</t>
+        </is>
+      </c>
+      <c r="X6" s="5" t="inlineStr">
+        <is>
+          <t>01А/2</t>
+        </is>
+      </c>
+      <c r="Y6" s="5" t="n"/>
+      <c r="Z6" s="5" t="n"/>
+      <c r="AA6" s="5" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="AB6" s="5" t="n"/>
+      <c r="AC6" s="5" t="n"/>
+      <c r="AD6" s="5" t="inlineStr">
+        <is>
+          <t>Вигаданий навчальний приклад; не є адресою реальної особи</t>
+        </is>
+      </c>
+      <c r="AE6" s="5" t="inlineStr">
+        <is>
+          <t>Україна</t>
+        </is>
+      </c>
+      <c r="AF6" s="5" t="inlineStr">
+        <is>
+          <t>Дніпропетровська</t>
+        </is>
+      </c>
+      <c r="AG6" s="5" t="inlineStr">
+        <is>
+          <t>Криворізький</t>
+        </is>
+      </c>
+      <c r="AH6" s="5" t="inlineStr">
+        <is>
+          <t>Криворізька</t>
+        </is>
+      </c>
+      <c r="AI6" s="5" t="inlineStr">
+        <is>
+          <t>Кривий Ріг</t>
+        </is>
+      </c>
+      <c r="AJ6" s="5" t="inlineStr">
+        <is>
+          <t>місто</t>
+        </is>
+      </c>
+      <c r="AK6" s="5" t="inlineStr">
+        <is>
+          <t>Бруно</t>
+        </is>
+      </c>
+      <c r="AL6" s="5" t="inlineStr">
+        <is>
+          <t>вулиця</t>
+        </is>
+      </c>
+      <c r="AM6" s="5" t="inlineStr">
+        <is>
+          <t>01А/2</t>
+        </is>
+      </c>
+      <c r="AN6" s="5" t="n"/>
+      <c r="AO6" s="5" t="n"/>
+      <c r="AP6" s="5" t="inlineStr">
+        <is>
+          <t>003</t>
+        </is>
+      </c>
+      <c r="AQ6" s="5" t="n"/>
+      <c r="AR6" s="5" t="n"/>
+      <c r="AS6" s="5" t="inlineStr">
+        <is>
+          <t>Вигаданий навчальний приклад; не є адресою реальної особи</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>version_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>structure_code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>valid_from</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>valid_to</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Назва версії</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Код структури</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Дата початку</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Дата завершення</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Навчальний штат 2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>training</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>